<commit_message>
Add 5-fold CV, logging, balanced split, evaluate_test_set update
</commit_message>
<xml_diff>
--- a/training_record.xlsx
+++ b/training_record.xlsx
@@ -1,28 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UserData\07大學教材\專題\Code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D5628F9-F434-495B-AA5F-67B7DF19D13B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A13AACB-A38E-49B0-8E51-249C7BAF6288}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="old" sheetId="1" r:id="rId1"/>
     <sheet name="v1(20260526)" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="v2(20260623)" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="82">
   <si>
     <t>model</t>
     <phoneticPr fontId="4" type="noConversion"/>
@@ -329,6 +329,26 @@
   </si>
   <si>
     <t>Test Classification Report</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>v1_F1</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>v1_F2</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>v1_F3</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>v1_F4</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>v1_F5</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -868,7 +888,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="107">
+  <cellXfs count="108">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1188,6 +1208,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="12" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="3" borderId="21" xfId="2" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4400,9 +4423,1024 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="B1:T28"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="27.6328125" customWidth="1"/>
+    <col min="9" max="9" width="27.54296875" customWidth="1"/>
+    <col min="16" max="16" width="27.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:20" ht="17.5" thickBot="1" x14ac:dyDescent="0.45"/>
+    <row r="2" spans="2:20" x14ac:dyDescent="0.4">
+      <c r="B2" s="65" t="s">
+        <v>77</v>
+      </c>
+      <c r="C2" s="66" t="s">
+        <v>47</v>
+      </c>
+      <c r="D2" s="66" t="s">
+        <v>48</v>
+      </c>
+      <c r="E2" s="66" t="s">
+        <v>49</v>
+      </c>
+      <c r="F2" s="67" t="s">
+        <v>50</v>
+      </c>
+      <c r="I2" s="65" t="s">
+        <v>78</v>
+      </c>
+      <c r="J2" s="66" t="s">
+        <v>47</v>
+      </c>
+      <c r="K2" s="66" t="s">
+        <v>48</v>
+      </c>
+      <c r="L2" s="66" t="s">
+        <v>49</v>
+      </c>
+      <c r="M2" s="67" t="s">
+        <v>50</v>
+      </c>
+      <c r="P2" s="65" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q2" s="66" t="s">
+        <v>47</v>
+      </c>
+      <c r="R2" s="66" t="s">
+        <v>48</v>
+      </c>
+      <c r="S2" s="66" t="s">
+        <v>49</v>
+      </c>
+      <c r="T2" s="67" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="2:20" x14ac:dyDescent="0.4">
+      <c r="B3" s="74" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3" s="75">
+        <v>0.75</v>
+      </c>
+      <c r="D3" s="75">
+        <v>0.81399999999999995</v>
+      </c>
+      <c r="E3" s="75">
+        <v>0.78</v>
+      </c>
+      <c r="F3" s="76">
+        <v>59</v>
+      </c>
+      <c r="I3" s="74" t="s">
+        <v>61</v>
+      </c>
+      <c r="J3" s="75">
+        <v>0.71</v>
+      </c>
+      <c r="K3" s="75">
+        <v>0.83099999999999996</v>
+      </c>
+      <c r="L3" s="75">
+        <v>0.76600000000000001</v>
+      </c>
+      <c r="M3" s="76">
+        <v>59</v>
+      </c>
+      <c r="P3" s="74" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q3" s="75">
+        <v>0.81799999999999995</v>
+      </c>
+      <c r="R3" s="75">
+        <v>0.76300000000000001</v>
+      </c>
+      <c r="S3" s="75">
+        <v>0.78900000000000003</v>
+      </c>
+      <c r="T3" s="76">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="2:20" x14ac:dyDescent="0.4">
+      <c r="B4" s="74" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="75">
+        <v>0.75</v>
+      </c>
+      <c r="D4" s="75">
+        <v>0.82799999999999996</v>
+      </c>
+      <c r="E4" s="75">
+        <v>0.78700000000000003</v>
+      </c>
+      <c r="F4" s="76">
+        <v>58</v>
+      </c>
+      <c r="I4" s="74" t="s">
+        <v>63</v>
+      </c>
+      <c r="J4" s="75">
+        <v>0.78300000000000003</v>
+      </c>
+      <c r="K4" s="75">
+        <v>0.81</v>
+      </c>
+      <c r="L4" s="75">
+        <v>0.79700000000000004</v>
+      </c>
+      <c r="M4" s="76">
+        <v>58</v>
+      </c>
+      <c r="P4" s="74" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q4" s="75">
+        <v>0.78800000000000003</v>
+      </c>
+      <c r="R4" s="75">
+        <v>0.89700000000000002</v>
+      </c>
+      <c r="S4" s="75">
+        <v>0.83899999999999997</v>
+      </c>
+      <c r="T4" s="76">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="2:20" x14ac:dyDescent="0.4">
+      <c r="B5" s="74" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="75">
+        <v>0.86799999999999999</v>
+      </c>
+      <c r="D5" s="75">
+        <v>0.78</v>
+      </c>
+      <c r="E5" s="75">
+        <v>0.82099999999999995</v>
+      </c>
+      <c r="F5" s="76">
+        <v>59</v>
+      </c>
+      <c r="I5" s="74" t="s">
+        <v>65</v>
+      </c>
+      <c r="J5" s="75">
+        <v>0.92</v>
+      </c>
+      <c r="K5" s="75">
+        <v>0.78</v>
+      </c>
+      <c r="L5" s="75">
+        <v>0.84399999999999997</v>
+      </c>
+      <c r="M5" s="76">
+        <v>59</v>
+      </c>
+      <c r="P5" s="74" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q5" s="75">
+        <v>0.84699999999999998</v>
+      </c>
+      <c r="R5" s="75">
+        <v>0.84699999999999998</v>
+      </c>
+      <c r="S5" s="75">
+        <v>0.84699999999999998</v>
+      </c>
+      <c r="T5" s="76">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="6" spans="2:20" x14ac:dyDescent="0.4">
+      <c r="B6" s="74" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6" s="75">
+        <v>0.879</v>
+      </c>
+      <c r="D6" s="75">
+        <v>0.85399999999999998</v>
+      </c>
+      <c r="E6" s="75">
+        <v>0.872</v>
+      </c>
+      <c r="F6" s="76">
+        <v>59</v>
+      </c>
+      <c r="I6" s="74" t="s">
+        <v>67</v>
+      </c>
+      <c r="J6" s="75">
+        <v>0.875</v>
+      </c>
+      <c r="K6" s="75">
+        <v>0.83099999999999996</v>
+      </c>
+      <c r="L6" s="75">
+        <v>0.85199999999999998</v>
+      </c>
+      <c r="M6" s="76">
+        <v>59</v>
+      </c>
+      <c r="P6" s="74" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q6" s="75">
+        <v>0.83599999999999997</v>
+      </c>
+      <c r="R6" s="75">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="S6" s="75">
+        <v>0.85</v>
+      </c>
+      <c r="T6" s="76">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7" spans="2:20" x14ac:dyDescent="0.4">
+      <c r="B7" s="74" t="s">
+        <v>68</v>
+      </c>
+      <c r="C7" s="75">
+        <v>0.92600000000000005</v>
+      </c>
+      <c r="D7" s="75">
+        <v>0.84699999999999998</v>
+      </c>
+      <c r="E7" s="75">
+        <v>0.88500000000000001</v>
+      </c>
+      <c r="F7" s="76">
+        <v>59</v>
+      </c>
+      <c r="I7" s="74" t="s">
+        <v>68</v>
+      </c>
+      <c r="J7" s="75">
+        <v>0.89500000000000002</v>
+      </c>
+      <c r="K7" s="75">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="L7" s="75">
+        <v>0.879</v>
+      </c>
+      <c r="M7" s="76">
+        <v>59</v>
+      </c>
+      <c r="P7" s="74" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q7" s="75">
+        <v>0.82</v>
+      </c>
+      <c r="R7" s="75">
+        <v>0.84699999999999998</v>
+      </c>
+      <c r="S7" s="75">
+        <v>0.83299999999999996</v>
+      </c>
+      <c r="T7" s="76">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8" spans="2:20" x14ac:dyDescent="0.4">
+      <c r="B8" s="74" t="s">
+        <v>69</v>
+      </c>
+      <c r="C8" s="75">
+        <v>0.81200000000000006</v>
+      </c>
+      <c r="D8" s="75">
+        <v>0.89700000000000002</v>
+      </c>
+      <c r="E8" s="75">
+        <v>0.85199999999999998</v>
+      </c>
+      <c r="F8" s="76">
+        <v>58</v>
+      </c>
+      <c r="I8" s="74" t="s">
+        <v>69</v>
+      </c>
+      <c r="J8" s="75">
+        <v>0.89800000000000002</v>
+      </c>
+      <c r="K8" s="75">
+        <v>0.91400000000000003</v>
+      </c>
+      <c r="L8" s="75">
+        <v>0.90600000000000003</v>
+      </c>
+      <c r="M8" s="76">
+        <v>58</v>
+      </c>
+      <c r="P8" s="74" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q8" s="75">
+        <v>0.90200000000000002</v>
+      </c>
+      <c r="R8" s="75">
+        <v>0.79300000000000004</v>
+      </c>
+      <c r="S8" s="75">
+        <v>0.84399999999999997</v>
+      </c>
+      <c r="T8" s="76">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" spans="2:20" x14ac:dyDescent="0.4">
+      <c r="B9" s="74" t="s">
+        <v>70</v>
+      </c>
+      <c r="C9" s="75">
+        <v>0.89100000000000001</v>
+      </c>
+      <c r="D9" s="75">
+        <v>0.83099999999999996</v>
+      </c>
+      <c r="E9" s="75">
+        <v>0.86</v>
+      </c>
+      <c r="F9" s="76">
+        <v>59</v>
+      </c>
+      <c r="I9" s="74" t="s">
+        <v>70</v>
+      </c>
+      <c r="J9" s="75">
+        <v>0.82799999999999996</v>
+      </c>
+      <c r="K9" s="75">
+        <v>0.89800000000000002</v>
+      </c>
+      <c r="L9" s="75">
+        <v>0.86199999999999999</v>
+      </c>
+      <c r="M9" s="76">
+        <v>59</v>
+      </c>
+      <c r="P9" s="74" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q9" s="75">
+        <v>0.79400000000000004</v>
+      </c>
+      <c r="R9" s="75">
+        <v>0.84699999999999998</v>
+      </c>
+      <c r="S9" s="75">
+        <v>0.82</v>
+      </c>
+      <c r="T9" s="76">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="2:20" x14ac:dyDescent="0.4">
+      <c r="B10" s="74" t="s">
+        <v>71</v>
+      </c>
+      <c r="C10" s="75">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="D10" s="75">
+        <v>0.879</v>
+      </c>
+      <c r="E10" s="75">
+        <v>0.872</v>
+      </c>
+      <c r="F10" s="76">
+        <v>58</v>
+      </c>
+      <c r="I10" s="74" t="s">
+        <v>71</v>
+      </c>
+      <c r="J10" s="75">
+        <v>0.90900000000000003</v>
+      </c>
+      <c r="K10" s="75">
+        <v>0.86199999999999999</v>
+      </c>
+      <c r="L10" s="75">
+        <v>0.88500000000000001</v>
+      </c>
+      <c r="M10" s="76">
+        <v>58</v>
+      </c>
+      <c r="P10" s="74" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q10" s="75">
+        <v>0.83099999999999996</v>
+      </c>
+      <c r="R10" s="75">
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="S10" s="75">
+        <v>0.83799999999999997</v>
+      </c>
+      <c r="T10" s="76">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="2:20" x14ac:dyDescent="0.4">
+      <c r="B11" s="74" t="s">
+        <v>72</v>
+      </c>
+      <c r="C11" s="75">
+        <v>0.94699999999999995</v>
+      </c>
+      <c r="D11" s="75">
+        <v>0.91500000000000004</v>
+      </c>
+      <c r="E11" s="75">
+        <v>0.93100000000000005</v>
+      </c>
+      <c r="F11" s="76">
+        <v>59</v>
+      </c>
+      <c r="I11" s="74" t="s">
+        <v>72</v>
+      </c>
+      <c r="J11" s="75">
+        <v>0.93100000000000005</v>
+      </c>
+      <c r="K11" s="75">
+        <v>0.91500000000000004</v>
+      </c>
+      <c r="L11" s="75">
+        <v>0.92300000000000004</v>
+      </c>
+      <c r="M11" s="76">
+        <v>59</v>
+      </c>
+      <c r="P11" s="74" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q11" s="75">
+        <v>0.96199999999999997</v>
+      </c>
+      <c r="R11" s="75">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="S11" s="75">
+        <v>0.91100000000000003</v>
+      </c>
+      <c r="T11" s="76">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="2:20" x14ac:dyDescent="0.4">
+      <c r="B12" s="96" t="s">
+        <v>73</v>
+      </c>
+      <c r="C12" s="97"/>
+      <c r="D12" s="97"/>
+      <c r="E12" s="97">
+        <v>0.85</v>
+      </c>
+      <c r="F12" s="98">
+        <v>528</v>
+      </c>
+      <c r="I12" s="96" t="s">
+        <v>73</v>
+      </c>
+      <c r="J12" s="97"/>
+      <c r="K12" s="97"/>
+      <c r="L12" s="97">
+        <v>0.85599999999999998</v>
+      </c>
+      <c r="M12" s="98">
+        <v>528</v>
+      </c>
+      <c r="P12" s="96" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q12" s="97"/>
+      <c r="R12" s="97"/>
+      <c r="S12" s="97">
+        <v>0.84099999999999997</v>
+      </c>
+      <c r="T12" s="98">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="13" spans="2:20" x14ac:dyDescent="0.4">
+      <c r="B13" s="99" t="s">
+        <v>74</v>
+      </c>
+      <c r="C13" s="75">
+        <v>0.85399999999999998</v>
+      </c>
+      <c r="D13" s="75">
+        <v>0.85</v>
+      </c>
+      <c r="E13" s="75">
+        <v>0.85099999999999998</v>
+      </c>
+      <c r="F13" s="76">
+        <v>528</v>
+      </c>
+      <c r="I13" s="99" t="s">
+        <v>74</v>
+      </c>
+      <c r="J13" s="75">
+        <v>0.86099999999999999</v>
+      </c>
+      <c r="K13" s="75">
+        <v>0.85599999999999998</v>
+      </c>
+      <c r="L13" s="75">
+        <v>0.85699999999999998</v>
+      </c>
+      <c r="M13" s="76">
+        <v>528</v>
+      </c>
+      <c r="P13" s="99" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q13" s="75">
+        <v>0.84399999999999997</v>
+      </c>
+      <c r="R13" s="75">
+        <v>0.84099999999999997</v>
+      </c>
+      <c r="S13" s="75">
+        <v>0.84099999999999997</v>
+      </c>
+      <c r="T13" s="76">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="14" spans="2:20" ht="17.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B14" s="100" t="s">
+        <v>75</v>
+      </c>
+      <c r="C14" s="101">
+        <v>0.85499999999999998</v>
+      </c>
+      <c r="D14" s="101">
+        <v>0.85</v>
+      </c>
+      <c r="E14" s="101">
+        <v>0.85099999999999998</v>
+      </c>
+      <c r="F14" s="102">
+        <v>528</v>
+      </c>
+      <c r="I14" s="100" t="s">
+        <v>75</v>
+      </c>
+      <c r="J14" s="101">
+        <v>0.86099999999999999</v>
+      </c>
+      <c r="K14" s="101">
+        <v>0.85599999999999998</v>
+      </c>
+      <c r="L14" s="101">
+        <v>0.85699999999999998</v>
+      </c>
+      <c r="M14" s="102">
+        <v>528</v>
+      </c>
+      <c r="P14" s="100" t="s">
+        <v>75</v>
+      </c>
+      <c r="Q14" s="101">
+        <v>0.84399999999999997</v>
+      </c>
+      <c r="R14" s="101">
+        <v>0.84099999999999997</v>
+      </c>
+      <c r="S14" s="101">
+        <v>0.84099999999999997</v>
+      </c>
+      <c r="T14" s="102">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="15" spans="2:20" ht="17.5" thickBot="1" x14ac:dyDescent="0.45"/>
+    <row r="16" spans="2:20" x14ac:dyDescent="0.4">
+      <c r="B16" s="65" t="s">
+        <v>80</v>
+      </c>
+      <c r="C16" s="66" t="s">
+        <v>47</v>
+      </c>
+      <c r="D16" s="66" t="s">
+        <v>48</v>
+      </c>
+      <c r="E16" s="66" t="s">
+        <v>49</v>
+      </c>
+      <c r="F16" s="67" t="s">
+        <v>50</v>
+      </c>
+      <c r="I16" s="65" t="s">
+        <v>81</v>
+      </c>
+      <c r="J16" s="66" t="s">
+        <v>47</v>
+      </c>
+      <c r="K16" s="66" t="s">
+        <v>48</v>
+      </c>
+      <c r="L16" s="66" t="s">
+        <v>49</v>
+      </c>
+      <c r="M16" s="67" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13" x14ac:dyDescent="0.4">
+      <c r="B17" s="74" t="s">
+        <v>61</v>
+      </c>
+      <c r="C17" s="75">
+        <v>0.78400000000000003</v>
+      </c>
+      <c r="D17" s="75">
+        <v>0.67800000000000005</v>
+      </c>
+      <c r="E17" s="75">
+        <v>0.72699999999999998</v>
+      </c>
+      <c r="F17" s="76">
+        <v>59</v>
+      </c>
+      <c r="I17" s="74" t="s">
+        <v>61</v>
+      </c>
+      <c r="J17" s="75">
+        <v>0.73799999999999999</v>
+      </c>
+      <c r="K17" s="75">
+        <v>0.81399999999999995</v>
+      </c>
+      <c r="L17" s="75">
+        <v>0.77400000000000002</v>
+      </c>
+      <c r="M17" s="76">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13" x14ac:dyDescent="0.4">
+      <c r="B18" s="74" t="s">
+        <v>63</v>
+      </c>
+      <c r="C18" s="75">
+        <v>0.77600000000000002</v>
+      </c>
+      <c r="D18" s="75">
+        <v>0.77600000000000002</v>
+      </c>
+      <c r="E18" s="75">
+        <v>0.77600000000000002</v>
+      </c>
+      <c r="F18" s="76">
+        <v>58</v>
+      </c>
+      <c r="I18" s="74" t="s">
+        <v>63</v>
+      </c>
+      <c r="J18" s="75">
+        <v>0.83599999999999997</v>
+      </c>
+      <c r="K18" s="75">
+        <v>0.79300000000000004</v>
+      </c>
+      <c r="L18" s="75">
+        <v>0.81399999999999995</v>
+      </c>
+      <c r="M18" s="76">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="19" spans="2:13" x14ac:dyDescent="0.4">
+      <c r="B19" s="74" t="s">
+        <v>65</v>
+      </c>
+      <c r="C19" s="75">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="D19" s="75">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="E19" s="75">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="F19" s="76">
+        <v>59</v>
+      </c>
+      <c r="I19" s="74" t="s">
+        <v>65</v>
+      </c>
+      <c r="J19" s="75">
+        <v>0.89100000000000001</v>
+      </c>
+      <c r="K19" s="75">
+        <v>0.83099999999999996</v>
+      </c>
+      <c r="L19" s="75">
+        <v>0.86</v>
+      </c>
+      <c r="M19" s="76">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13" x14ac:dyDescent="0.4">
+      <c r="B20" s="74" t="s">
+        <v>67</v>
+      </c>
+      <c r="C20" s="75">
+        <v>0.80600000000000005</v>
+      </c>
+      <c r="D20" s="75">
+        <v>0.84699999999999998</v>
+      </c>
+      <c r="E20" s="75">
+        <v>0.82599999999999996</v>
+      </c>
+      <c r="F20" s="76">
+        <v>59</v>
+      </c>
+      <c r="I20" s="74" t="s">
+        <v>67</v>
+      </c>
+      <c r="J20" s="75">
+        <v>0.85199999999999998</v>
+      </c>
+      <c r="K20" s="75">
+        <v>0.88100000000000001</v>
+      </c>
+      <c r="L20" s="75">
+        <v>0.86699999999999999</v>
+      </c>
+      <c r="M20" s="76">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="21" spans="2:13" x14ac:dyDescent="0.4">
+      <c r="B21" s="74" t="s">
+        <v>68</v>
+      </c>
+      <c r="C21" s="75">
+        <v>0.90900000000000003</v>
+      </c>
+      <c r="D21" s="75">
+        <v>0.84699999999999998</v>
+      </c>
+      <c r="E21" s="75">
+        <v>0.877</v>
+      </c>
+      <c r="F21" s="76">
+        <v>59</v>
+      </c>
+      <c r="I21" s="74" t="s">
+        <v>68</v>
+      </c>
+      <c r="J21" s="75">
+        <v>0.86199999999999999</v>
+      </c>
+      <c r="K21" s="75">
+        <v>0.84699999999999998</v>
+      </c>
+      <c r="L21" s="75">
+        <v>0.85499999999999998</v>
+      </c>
+      <c r="M21" s="76">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="22" spans="2:13" x14ac:dyDescent="0.4">
+      <c r="B22" s="74" t="s">
+        <v>69</v>
+      </c>
+      <c r="C22" s="75">
+        <v>0.84699999999999998</v>
+      </c>
+      <c r="D22" s="75">
+        <v>0.86199999999999999</v>
+      </c>
+      <c r="E22" s="75">
+        <v>0.85499999999999998</v>
+      </c>
+      <c r="F22" s="76">
+        <v>59</v>
+      </c>
+      <c r="I22" s="74" t="s">
+        <v>69</v>
+      </c>
+      <c r="J22" s="75">
+        <v>0.873</v>
+      </c>
+      <c r="K22" s="75">
+        <v>0.82799999999999996</v>
+      </c>
+      <c r="L22" s="75">
+        <v>0.85</v>
+      </c>
+      <c r="M22" s="76">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="23" spans="2:13" x14ac:dyDescent="0.4">
+      <c r="B23" s="74" t="s">
+        <v>70</v>
+      </c>
+      <c r="C23" s="75">
+        <v>0.8</v>
+      </c>
+      <c r="D23" s="75">
+        <v>0.88100000000000001</v>
+      </c>
+      <c r="E23" s="75">
+        <v>0.83899999999999997</v>
+      </c>
+      <c r="F23" s="76">
+        <v>59</v>
+      </c>
+      <c r="I23" s="74" t="s">
+        <v>70</v>
+      </c>
+      <c r="J23" s="75">
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="K23" s="75">
+        <v>0.83099999999999996</v>
+      </c>
+      <c r="L23" s="75">
+        <v>0.83799999999999997</v>
+      </c>
+      <c r="M23" s="76">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="24" spans="2:13" x14ac:dyDescent="0.4">
+      <c r="B24" s="74" t="s">
+        <v>71</v>
+      </c>
+      <c r="C24" s="75">
+        <v>0.89700000000000002</v>
+      </c>
+      <c r="D24" s="75">
+        <v>0.89700000000000002</v>
+      </c>
+      <c r="E24" s="75">
+        <v>0.89700000000000002</v>
+      </c>
+      <c r="F24" s="76">
+        <v>58</v>
+      </c>
+      <c r="I24" s="74" t="s">
+        <v>71</v>
+      </c>
+      <c r="J24" s="75">
+        <v>0.81499999999999995</v>
+      </c>
+      <c r="K24" s="75">
+        <v>0.91400000000000003</v>
+      </c>
+      <c r="L24" s="75">
+        <v>0.86199999999999999</v>
+      </c>
+      <c r="M24" s="76">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="25" spans="2:13" x14ac:dyDescent="0.4">
+      <c r="B25" s="74" t="s">
+        <v>72</v>
+      </c>
+      <c r="C25" s="75">
+        <v>0.88500000000000001</v>
+      </c>
+      <c r="D25" s="75">
+        <v>0.91500000000000004</v>
+      </c>
+      <c r="E25" s="75">
+        <v>0.9</v>
+      </c>
+      <c r="F25" s="76">
+        <v>59</v>
+      </c>
+      <c r="I25" s="74" t="s">
+        <v>72</v>
+      </c>
+      <c r="J25" s="75">
+        <v>0.94599999999999995</v>
+      </c>
+      <c r="K25" s="75">
+        <v>0.89800000000000002</v>
+      </c>
+      <c r="L25" s="75">
+        <v>0.92200000000000004</v>
+      </c>
+      <c r="M25" s="76">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="26" spans="2:13" x14ac:dyDescent="0.4">
+      <c r="B26" s="96" t="s">
+        <v>73</v>
+      </c>
+      <c r="C26" s="97"/>
+      <c r="D26" s="97"/>
+      <c r="E26" s="97">
+        <v>0.84099999999999997</v>
+      </c>
+      <c r="F26" s="98">
+        <v>528</v>
+      </c>
+      <c r="I26" s="96" t="s">
+        <v>73</v>
+      </c>
+      <c r="J26" s="97"/>
+      <c r="K26" s="97"/>
+      <c r="L26" s="97">
+        <v>0.84799999999999998</v>
+      </c>
+      <c r="M26" s="98">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="27" spans="2:13" x14ac:dyDescent="0.4">
+      <c r="B27" s="99" t="s">
+        <v>74</v>
+      </c>
+      <c r="C27" s="75">
+        <v>0.84099999999999997</v>
+      </c>
+      <c r="D27" s="75">
+        <v>0.84099999999999997</v>
+      </c>
+      <c r="E27" s="75">
+        <v>0.84</v>
+      </c>
+      <c r="F27" s="76">
+        <v>528</v>
+      </c>
+      <c r="I27" s="99" t="s">
+        <v>74</v>
+      </c>
+      <c r="J27" s="75">
+        <v>0.85099999999999998</v>
+      </c>
+      <c r="K27" s="75">
+        <v>0.84799999999999998</v>
+      </c>
+      <c r="L27" s="75">
+        <v>0.84899999999999998</v>
+      </c>
+      <c r="M27" s="76">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="28" spans="2:13" ht="17.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B28" s="100" t="s">
+        <v>75</v>
+      </c>
+      <c r="C28" s="101">
+        <v>0.84099999999999997</v>
+      </c>
+      <c r="D28" s="101">
+        <v>0.84099999999999997</v>
+      </c>
+      <c r="E28" s="107">
+        <v>0.84</v>
+      </c>
+      <c r="F28" s="102">
+        <v>528</v>
+      </c>
+      <c r="I28" s="100" t="s">
+        <v>75</v>
+      </c>
+      <c r="J28" s="101">
+        <v>0.85099999999999998</v>
+      </c>
+      <c r="K28" s="101">
+        <v>0.84799999999999998</v>
+      </c>
+      <c r="L28" s="101">
+        <v>0.84899999999999998</v>
+      </c>
+      <c r="M28" s="102">
+        <v>528</v>
+      </c>
+    </row>
+  </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>